<commit_message>
DOC:Actualización de la planificacion temporal
</commit_message>
<xml_diff>
--- a/A-Documentacion/B-Elaboracion/Iteracion1-24_09-al-16_10/eGraduados_Elaboracion_Iteracion1_PlanificacionTemporal.xlsx
+++ b/A-Documentacion/B-Elaboracion/Iteracion1-24_09-al-16_10/eGraduados_Elaboracion_Iteracion1_PlanificacionTemporal.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Usuario\Documents\eGraduados\A-Documentacion\B-Elaboracion\Iteracion1\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Usuario\Documents\eGraduados\A-Documentacion\B-Elaboracion\Iteracion1-24_09-al-16_10\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B19A53AB-4B34-4328-915E-390C82D22AA2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{594B53B9-20BD-49DF-BA75-88180552EDB9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{C157A7F2-5B1B-4E06-B43B-1F6A14E9BE8B}"/>
+    <workbookView xWindow="10245" yWindow="0" windowWidth="10245" windowHeight="10920" xr2:uid="{C157A7F2-5B1B-4E06-B43B-1F6A14E9BE8B}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -107,9 +107,6 @@
     <t>Planificaicón temporal eGraduados - Elaboracion Iteracion 1 - 24/09 al 16/10</t>
   </si>
   <si>
-    <t>Realizar diseño lógico de la BBDD</t>
-  </si>
-  <si>
     <t>Realizar normalización de la BBDD</t>
   </si>
   <si>
@@ -135,6 +132,9 @@
   </si>
   <si>
     <t>5;10</t>
+  </si>
+  <si>
+    <t>Realizar diseño conceptual y lógico de la BBDD</t>
   </si>
 </sst>
 </file>
@@ -218,20 +218,18 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="16" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -580,16 +578,16 @@
   </cols>
   <sheetData>
     <row r="3" spans="3:10" x14ac:dyDescent="0.25">
-      <c r="C3" s="5" t="s">
+      <c r="C3" s="8" t="s">
         <v>21</v>
       </c>
-      <c r="D3" s="5"/>
-      <c r="E3" s="5"/>
-      <c r="F3" s="5"/>
-      <c r="G3" s="5"/>
-      <c r="H3" s="5"/>
-      <c r="I3" s="5"/>
-      <c r="J3" s="5"/>
+      <c r="D3" s="8"/>
+      <c r="E3" s="8"/>
+      <c r="F3" s="8"/>
+      <c r="G3" s="8"/>
+      <c r="H3" s="8"/>
+      <c r="I3" s="8"/>
+      <c r="J3" s="8"/>
     </row>
     <row r="4" spans="3:10" x14ac:dyDescent="0.25">
       <c r="C4" s="4" t="s">
@@ -619,9 +617,9 @@
     </row>
     <row r="5" spans="3:10" x14ac:dyDescent="0.25">
       <c r="C5" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="D5" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="D5" s="6" t="s">
         <v>9</v>
       </c>
       <c r="E5" s="2" t="s">
@@ -635,11 +633,11 @@
       </c>
       <c r="H5" s="1"/>
       <c r="I5" s="1"/>
-      <c r="J5" s="6"/>
+      <c r="J5" s="5"/>
     </row>
     <row r="6" spans="3:10" x14ac:dyDescent="0.25">
       <c r="C6" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D6" s="3" t="s">
         <v>8</v>
@@ -655,11 +653,11 @@
       </c>
       <c r="H6" s="1"/>
       <c r="I6" s="1"/>
-      <c r="J6" s="6"/>
+      <c r="J6" s="5"/>
     </row>
     <row r="7" spans="3:10" x14ac:dyDescent="0.25">
       <c r="C7" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="D7" s="1" t="s">
         <v>11</v>
@@ -675,9 +673,9 @@
       </c>
       <c r="H7" s="1"/>
       <c r="I7" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="J7" s="6"/>
+        <v>26</v>
+      </c>
+      <c r="J7" s="5"/>
     </row>
     <row r="8" spans="3:10" x14ac:dyDescent="0.25">
       <c r="C8" s="1">
@@ -717,13 +715,13 @@
       </c>
       <c r="H9" s="1"/>
       <c r="I9" s="1"/>
-      <c r="J9" s="6"/>
+      <c r="J9" s="5"/>
     </row>
     <row r="10" spans="3:10" x14ac:dyDescent="0.25">
       <c r="C10" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="D10" s="7" t="s">
+      <c r="D10" s="6" t="s">
         <v>12</v>
       </c>
       <c r="E10" s="2">
@@ -737,13 +735,13 @@
       </c>
       <c r="H10" s="1"/>
       <c r="I10" s="1"/>
-      <c r="J10" s="6"/>
+      <c r="J10" s="5"/>
     </row>
     <row r="11" spans="3:10" x14ac:dyDescent="0.25">
       <c r="C11" s="1">
         <v>2</v>
       </c>
-      <c r="D11" s="7" t="s">
+      <c r="D11" s="6" t="s">
         <v>14</v>
       </c>
       <c r="E11" s="2">
@@ -757,7 +755,7 @@
       </c>
       <c r="H11" s="1"/>
       <c r="I11" s="1"/>
-      <c r="J11" s="6"/>
+      <c r="J11" s="5"/>
     </row>
     <row r="12" spans="3:10" x14ac:dyDescent="0.25">
       <c r="C12" s="1">
@@ -779,14 +777,14 @@
       <c r="I12" s="1">
         <v>1</v>
       </c>
-      <c r="J12" s="6"/>
+      <c r="J12" s="5"/>
     </row>
     <row r="13" spans="3:10" x14ac:dyDescent="0.25">
       <c r="C13" s="1">
         <v>4</v>
       </c>
       <c r="D13" s="3" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="E13" s="2">
         <v>46302</v>
@@ -801,13 +799,13 @@
       <c r="I13" s="1">
         <v>1</v>
       </c>
-      <c r="J13" s="6"/>
+      <c r="J13" s="5"/>
     </row>
     <row r="14" spans="3:10" x14ac:dyDescent="0.25">
       <c r="C14" s="1">
         <v>5</v>
       </c>
-      <c r="D14" s="8" t="s">
+      <c r="D14" s="7" t="s">
         <v>18</v>
       </c>
       <c r="E14" s="2">
@@ -823,7 +821,7 @@
       <c r="I14" s="1">
         <v>1</v>
       </c>
-      <c r="J14" s="6"/>
+      <c r="J14" s="5"/>
     </row>
     <row r="15" spans="3:10" x14ac:dyDescent="0.25">
       <c r="C15" s="1">
@@ -863,7 +861,7 @@
       </c>
       <c r="H16" s="1"/>
       <c r="I16" s="1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="J16" s="1"/>
     </row>
@@ -872,7 +870,7 @@
         <v>8</v>
       </c>
       <c r="D17" s="3" t="s">
-        <v>22</v>
+        <v>31</v>
       </c>
       <c r="E17" s="2">
         <v>46307</v>
@@ -892,7 +890,7 @@
         <v>9</v>
       </c>
       <c r="D18" s="3" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E18" s="2">
         <v>46310</v>
@@ -914,7 +912,7 @@
         <v>10</v>
       </c>
       <c r="D19" s="3" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="E19" s="2">
         <v>46311</v>
@@ -932,11 +930,11 @@
       <c r="J19" s="1"/>
     </row>
     <row r="20" spans="3:10" x14ac:dyDescent="0.25">
-      <c r="C20" s="9">
+      <c r="C20" s="1">
         <v>11</v>
       </c>
-      <c r="D20" s="10" t="s">
-        <v>25</v>
+      <c r="D20" s="7" t="s">
+        <v>24</v>
       </c>
       <c r="E20" s="2">
         <v>46311</v>
@@ -944,12 +942,12 @@
       <c r="F20" s="2">
         <v>46311</v>
       </c>
-      <c r="G20" s="9">
+      <c r="G20" s="1">
         <v>2</v>
       </c>
       <c r="H20" s="1"/>
       <c r="I20" s="1" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="J20" s="1"/>
     </row>

</xml_diff>